<commit_message>
Update: Refined ETL pipeline and updated mapping documentation
</commit_message>
<xml_diff>
--- a/docs/Book_DWH_mapping.xlsx
+++ b/docs/Book_DWH_mapping.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\DEPI\projects\Book_DWH\mapping\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\DEPI\projects\Book_DWH\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E69FD484-AEDD-48BE-BAC7-D9D843D5B4FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26B39405-3FE6-4D89-AED0-164B42D42C60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="13056" xr2:uid="{2D03D3A6-4D81-4ED0-BDBF-1F56EA5338E9}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{2D03D3A6-4D81-4ED0-BDBF-1F56EA5338E9}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -58,7 +58,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="64">
   <si>
     <t>DIM_Customer</t>
   </si>
@@ -235,6 +235,21 @@
   </si>
   <si>
     <t xml:space="preserve">int </t>
+  </si>
+  <si>
+    <t>Dim_Author</t>
+  </si>
+  <si>
+    <t>Author_SK</t>
+  </si>
+  <si>
+    <t>Author_ID</t>
+  </si>
+  <si>
+    <t>Bridge_Book_Author</t>
+  </si>
+  <si>
+    <t>int(PK)</t>
   </si>
 </sst>
 </file>
@@ -674,7 +689,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FCDBE1E5-0CAD-4400-A298-947A3F6C3EE0}">
-  <dimension ref="A1:F45"/>
+  <dimension ref="A1:F62"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="41.5546875" customWidth="1"/>
@@ -912,7 +927,7 @@
     </row>
     <row r="25" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A25" s="7" t="s">
-        <v>34</v>
+        <v>59</v>
       </c>
       <c r="B25" s="8"/>
       <c r="C25" s="8"/>
@@ -934,7 +949,7 @@
     </row>
     <row r="27" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A27" s="1" t="s">
-        <v>35</v>
+        <v>60</v>
       </c>
       <c r="B27" s="2" t="s">
         <v>6</v>
@@ -952,221 +967,338 @@
     </row>
     <row r="28" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A28" s="1" t="s">
-        <v>36</v>
+        <v>61</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>6</v>
+        <v>22</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>6</v>
+        <v>23</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>42</v>
+        <v>19</v>
       </c>
     </row>
     <row r="29" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A29" s="1" t="s">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>6</v>
+        <v>22</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>6</v>
+        <v>24</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="30" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A30" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="B30" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C30" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D30" s="2" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="31" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A31" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="B31" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C31" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D31" s="2" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="32" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A32" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="B32" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C32" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D32" s="2" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A33" s="4"/>
-      <c r="B33" s="4"/>
-      <c r="C33" s="4"/>
-      <c r="D33" s="4"/>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A33" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="B33" s="8"/>
+      <c r="C33" s="8"/>
+      <c r="D33" s="8"/>
+    </row>
+    <row r="34" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A34" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C34" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D34" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A35" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C35" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D35" s="2" t="s">
+        <v>41</v>
+      </c>
     </row>
     <row r="36" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A36" s="7" t="s">
-        <v>57</v>
-      </c>
-      <c r="B36" s="7"/>
-      <c r="C36" s="7"/>
-      <c r="D36" s="7"/>
-    </row>
-    <row r="37" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A37" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B37" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C37" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="D37" s="1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="38" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A38" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="B38" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C38" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D38" s="2" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="39" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A39" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="B39" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="C39" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="D39" s="2" t="s">
-        <v>53</v>
+      <c r="A36" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="D36" s="2" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="40" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A40" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B40" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="C40" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="D40" s="2" t="s">
-        <v>53</v>
-      </c>
+      <c r="A40" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="B40" s="5"/>
+      <c r="C40" s="5"/>
+      <c r="D40" s="5"/>
     </row>
     <row r="41" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A41" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="B41" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="C41" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="D41" s="2" t="s">
-        <v>53</v>
+        <v>1</v>
+      </c>
+      <c r="B41" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C41" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D41" s="1" t="s">
+        <v>4</v>
       </c>
     </row>
     <row r="42" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A42" s="1" t="s">
-        <v>48</v>
+        <v>35</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>45</v>
+        <v>6</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>49</v>
+        <v>6</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
     </row>
     <row r="43" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A43" s="1" t="s">
-        <v>50</v>
+        <v>36</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>47</v>
+        <v>6</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>50</v>
+        <v>6</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>19</v>
+        <v>42</v>
       </c>
     </row>
     <row r="44" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A44" s="1" t="s">
-        <v>51</v>
+        <v>37</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>47</v>
+        <v>6</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>31</v>
+        <v>6</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>33</v>
+        <v>19</v>
       </c>
     </row>
     <row r="45" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A45" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B45" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C45" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D45" s="2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A46" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="B46" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C46" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D46" s="2" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A47" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B47" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C47" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D47" s="2" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A48" s="4"/>
+      <c r="B48" s="4"/>
+      <c r="C48" s="4"/>
+      <c r="D48" s="4"/>
+    </row>
+    <row r="53" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A53" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="B53" s="5"/>
+      <c r="C53" s="5"/>
+      <c r="D53" s="5"/>
+    </row>
+    <row r="54" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A54" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B54" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C54" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D54" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A55" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B55" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C55" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D55" s="2" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A56" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B56" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C56" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="D56" s="2" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A57" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B57" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C57" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D57" s="2" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A58" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B58" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="C58" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="D58" s="2" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A59" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="B59" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C59" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D59" s="2" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A60" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="B60" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="C60" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="D60" s="2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A61" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="B61" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="C61" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D61" s="2" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A62" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="B45" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C45" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D45" s="2" t="s">
+      <c r="B62" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C62" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D62" s="2" t="s">
         <v>54</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="6">
+    <mergeCell ref="A25:D25"/>
+    <mergeCell ref="A33:D33"/>
+    <mergeCell ref="A40:D40"/>
+    <mergeCell ref="A53:D53"/>
     <mergeCell ref="A13:D13"/>
     <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A25:D25"/>
-    <mergeCell ref="A36:D36"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>